<commit_message>
feat(call-tracking): add email column to call logs, uploads, and exports
</commit_message>
<xml_diff>
--- a/public/templates/Call_Log_Template.xlsx
+++ b/public/templates/Call_Log_Template.xlsx
@@ -490,7 +490,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
@@ -554,7 +554,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Emailed?</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">

</xml_diff>